<commit_message>
up to generating quarto and manuscript draft
</commit_message>
<xml_diff>
--- a/code/CO_capsule_infos.xlsx
+++ b/code/CO_capsule_infos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute-my.sharepoint.com/personal/jinho_kim_alleninstitute_org/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="481" documentId="8_{0A446674-3EF5-E34C-A612-F2F4FA538D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7116FF9-8723-814A-8CA9-A414CC74E870}"/>
+  <xr:revisionPtr revIDLastSave="500" documentId="8_{0A446674-3EF5-E34C-A612-F2F4FA538D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A754E94-3F4F-BE4B-BA63-C0B21D7C9074}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C0A60769-E7A5-2E47-AEAD-530C78EEC6C4}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="236">
   <si>
     <t>capsule name</t>
   </si>
@@ -379,9 +379,6 @@
     <t>ROICat</t>
   </si>
   <si>
-    <t>all processed ophys data assets</t>
-  </si>
-  <si>
     <t>Running ROICaT for cross-session matching</t>
   </si>
   <si>
@@ -400,9 +397,6 @@
     <t>single-cell-zdrift-qc</t>
   </si>
   <si>
-    <t>Ophys processed data asset (single session)</t>
-  </si>
-  <si>
     <t>https://codeocean.allenneuraldynamics.org/capsule/8634983/tree</t>
   </si>
   <si>
@@ -502,9 +496,6 @@
     <t>c975fe83-f91d-457e-9e28-596e1e551790</t>
   </si>
   <si>
-    <t>Ophys processed data asset with z-stack (can be searched via docDB and s3)</t>
-  </si>
-  <si>
     <t>Cortical z-stack registration - needs update for expansion across plane-to-plane registration</t>
   </si>
   <si>
@@ -718,12 +709,6 @@
     <t>8935ac9e-7c9c-474a-ab30-e2cb8af7c341</t>
   </si>
   <si>
-    <t>3DFISH-autocoreg</t>
-  </si>
-  <si>
-    <t>3DFISH-autocoreg-qced</t>
-  </si>
-  <si>
     <t>HCR processed (R1); HCR-ROI-label; cortical-zstack-registration; cortical-zstack-segmentation</t>
   </si>
   <si>
@@ -731,6 +716,36 @@
   </si>
   <si>
     <t>Running automatic co-registration between 2p czstack and 3D FISH and generate pre_coreg_table.csv</t>
+  </si>
+  <si>
+    <t>Jinho_pipeline_monitor_2p-3DFISH-autocoreg</t>
+  </si>
+  <si>
+    <t>https://codeocean.allenneuraldynamics.org/capsule/1213311/tree</t>
+  </si>
+  <si>
+    <t>https://github.com/AllenNeuralDynamics/Jinho_pipeline-monitor_2p-3DFISH-autocoreg</t>
+  </si>
+  <si>
+    <t>efa9a7b1-f53a-4c82-833e-9b7cec69570a</t>
+  </si>
+  <si>
+    <t>ophys processed data</t>
+  </si>
+  <si>
+    <t>ophys processed data asset with cortical z-stack</t>
+  </si>
+  <si>
+    <t>ophys processed data asset (single session)</t>
+  </si>
+  <si>
+    <t>all processed ophys data assets from one mouse</t>
+  </si>
+  <si>
+    <t>2p-3DFISH-autocoreg</t>
+  </si>
+  <si>
+    <t>2p-3DFISH-autocoreg-qced</t>
   </si>
 </sst>
 </file>
@@ -775,10 +790,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1114,7 +1128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E2BDC0-D015-9444-B204-785BF3CFBE5E}">
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
@@ -1301,6 +1315,9 @@
       <c r="G7" t="s">
         <v>41</v>
       </c>
+      <c r="J7" t="s">
+        <v>144</v>
+      </c>
       <c r="M7" t="s">
         <v>49</v>
       </c>
@@ -1356,10 +1373,10 @@
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>53</v>
@@ -1394,10 +1411,10 @@
         <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>61</v>
@@ -1423,10 +1440,10 @@
         <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>62</v>
@@ -1452,28 +1469,28 @@
         <v>33</v>
       </c>
       <c r="D13" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>221</v>
-      </c>
       <c r="F13" s="1" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="G13" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H13" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="I13" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="J13" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="M13" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
@@ -1484,51 +1501,48 @@
         <v>33</v>
       </c>
       <c r="D14" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="G14" t="s">
+        <v>222</v>
+      </c>
+      <c r="H14" t="s">
+        <v>235</v>
+      </c>
+      <c r="I14" t="s">
+        <v>235</v>
+      </c>
+      <c r="J14" t="s">
+        <v>234</v>
+      </c>
+      <c r="M14" t="s">
         <v>224</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="G14" t="s">
-        <v>225</v>
-      </c>
-      <c r="H14" t="s">
-        <v>227</v>
-      </c>
-      <c r="I14" t="s">
-        <v>227</v>
-      </c>
-      <c r="J14" t="s">
-        <v>226</v>
-      </c>
-      <c r="M14" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" t="s">
-        <v>37</v>
+        <v>226</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>228</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>63</v>
+        <v>227</v>
       </c>
       <c r="G15" t="s">
-        <v>65</v>
-      </c>
-      <c r="M15" t="s">
-        <v>66</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -1536,45 +1550,45 @@
         <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="M16" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
         <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
         <v>37</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G17" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="M17" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -1585,67 +1599,73 @@
         <v>33</v>
       </c>
       <c r="D18" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>79</v>
+        <v>72</v>
+      </c>
+      <c r="E18" t="s">
+        <v>37</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="M18" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D19" t="s">
-        <v>90</v>
-      </c>
-      <c r="E19" t="s">
-        <v>37</v>
+        <v>77</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="M19" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>94</v>
+        <v>43</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" t="s">
+        <v>92</v>
+      </c>
+      <c r="M20" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>96</v>
+        <v>14</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -1656,91 +1676,76 @@
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>99</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
+      </c>
+      <c r="E22" t="s">
+        <v>37</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>102</v>
-      </c>
-      <c r="E23" t="s">
-        <v>37</v>
+        <v>99</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="G23" t="s">
-        <v>103</v>
-      </c>
-      <c r="M23" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D24" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E24" t="s">
         <v>37</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G24" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="M24" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E25" t="s">
         <v>37</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G25" t="s">
-        <v>111</v>
-      </c>
-      <c r="H25" t="s">
-        <v>112</v>
-      </c>
-      <c r="I25" t="s">
-        <v>112</v>
-      </c>
-      <c r="J25" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="M25" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
@@ -1751,129 +1756,129 @@
         <v>33</v>
       </c>
       <c r="D26" t="s">
-        <v>116</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G26" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H26" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="I26" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="J26" t="s">
-        <v>120</v>
+        <v>233</v>
       </c>
       <c r="M26" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
         <v>33</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="G27" t="s">
-        <v>124</v>
+        <v>117</v>
+      </c>
+      <c r="H27" t="s">
+        <v>118</v>
+      </c>
+      <c r="I27" t="s">
+        <v>118</v>
+      </c>
+      <c r="J27" t="s">
+        <v>232</v>
       </c>
       <c r="M27" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="C28" t="s">
         <v>33</v>
       </c>
       <c r="D28" t="s">
-        <v>127</v>
-      </c>
-      <c r="E28" t="s">
-        <v>37</v>
+        <v>120</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="G28" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="M28" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>43</v>
+        <v>126</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D29" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E29" t="s">
         <v>37</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="G29" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="M29" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C30" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D30" t="s">
-        <v>136</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
+      </c>
+      <c r="E30" t="s">
+        <v>37</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="G30" t="s">
-        <v>138</v>
-      </c>
-      <c r="H30" t="s">
-        <v>139</v>
-      </c>
-      <c r="I30" t="s">
-        <v>139</v>
-      </c>
-      <c r="J30" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="M30" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
@@ -1884,34 +1889,28 @@
         <v>33</v>
       </c>
       <c r="D31" t="s">
-        <v>143</v>
-      </c>
-      <c r="E31" t="s">
-        <v>37</v>
+        <v>134</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="G31" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="H31" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="I31" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="J31" t="s">
-        <v>146</v>
-      </c>
-      <c r="K31" t="s">
-        <v>147</v>
-      </c>
-      <c r="L31" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="M31" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
@@ -1922,28 +1921,34 @@
         <v>33</v>
       </c>
       <c r="D32" t="s">
-        <v>151</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>152</v>
+        <v>141</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G32" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="H32" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I32" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="J32" t="s">
-        <v>154</v>
+        <v>144</v>
+      </c>
+      <c r="K32" t="s">
+        <v>145</v>
+      </c>
+      <c r="L32" t="s">
+        <v>146</v>
       </c>
       <c r="M32" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
@@ -1954,51 +1959,54 @@
         <v>33</v>
       </c>
       <c r="D33" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="G33" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>138</v>
       </c>
       <c r="I33" t="s">
-        <v>174</v>
+        <v>138</v>
+      </c>
+      <c r="J33" t="s">
+        <v>231</v>
+      </c>
+      <c r="M33" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
         <v>33</v>
       </c>
       <c r="D34" t="s">
-        <v>160</v>
-      </c>
-      <c r="E34" t="s">
-        <v>37</v>
+        <v>154</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="G34" t="s">
-        <v>161</v>
+        <v>170</v>
+      </c>
+      <c r="H34" t="s">
+        <v>172</v>
       </c>
       <c r="I34" t="s">
-        <v>162</v>
-      </c>
-      <c r="J34" t="s">
-        <v>172</v>
-      </c>
-      <c r="M34" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
@@ -2009,204 +2017,195 @@
         <v>33</v>
       </c>
       <c r="D35" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="E35" t="s">
         <v>37</v>
       </c>
       <c r="F35" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G35" t="s">
+        <v>158</v>
+      </c>
+      <c r="I35" t="s">
+        <v>159</v>
+      </c>
+      <c r="J35" t="s">
         <v>169</v>
       </c>
-      <c r="G35" t="s">
-        <v>171</v>
-      </c>
-      <c r="I35" t="s">
-        <v>162</v>
+      <c r="M35" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C36" t="s">
         <v>33</v>
       </c>
       <c r="D36" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E36" t="s">
         <v>37</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G36" t="s">
-        <v>165</v>
-      </c>
-      <c r="H36" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I36" t="s">
-        <v>166</v>
-      </c>
-      <c r="J36" t="s">
-        <v>146</v>
-      </c>
-      <c r="M36" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
         <v>33</v>
       </c>
       <c r="D37" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="E37" t="s">
         <v>37</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="G37" t="s">
-        <v>178</v>
+        <v>162</v>
+      </c>
+      <c r="H37" t="s">
+        <v>163</v>
+      </c>
+      <c r="I37" t="s">
+        <v>163</v>
+      </c>
+      <c r="J37" t="s">
+        <v>144</v>
       </c>
       <c r="M37" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
       </c>
       <c r="D38" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E38" t="s">
         <v>37</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="G38" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="M38" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
       </c>
       <c r="D39" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E39" t="s">
         <v>37</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="G39" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="M39" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
       </c>
       <c r="D40" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="E40" t="s">
         <v>37</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="G40" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="M40" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
       <c r="C41" t="s">
         <v>33</v>
       </c>
       <c r="D41" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="E41" t="s">
         <v>37</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G41" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="M41" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C42" t="s">
         <v>33</v>
       </c>
       <c r="D42" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E42" t="s">
         <v>37</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G42" t="s">
-        <v>197</v>
-      </c>
-      <c r="H42" t="s">
-        <v>202</v>
-      </c>
-      <c r="I42" t="s">
-        <v>202</v>
-      </c>
-      <c r="J42" t="s">
-        <v>203</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="L42" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="M42" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
@@ -2214,45 +2213,86 @@
         <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D43" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E43" t="s">
         <v>37</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="G43" t="s">
-        <v>206</v>
+        <v>194</v>
+      </c>
+      <c r="H43" t="s">
+        <v>199</v>
+      </c>
+      <c r="I43" t="s">
+        <v>199</v>
+      </c>
+      <c r="J43" t="s">
+        <v>200</v>
+      </c>
+      <c r="K43" t="s">
+        <v>196</v>
+      </c>
+      <c r="L43" t="s">
+        <v>197</v>
       </c>
       <c r="M43" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>128</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D44" t="s">
+        <v>202</v>
+      </c>
+      <c r="E44" t="s">
+        <v>37</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44" t="s">
+        <v>203</v>
+      </c>
+      <c r="J44" t="s">
+        <v>230</v>
+      </c>
+      <c r="M44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>126</v>
+      </c>
+      <c r="C45" t="s">
+        <v>33</v>
+      </c>
+      <c r="D45" t="s">
+        <v>205</v>
+      </c>
+      <c r="E45" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G45" t="s">
+        <v>207</v>
+      </c>
+      <c r="M45" t="s">
         <v>208</v>
-      </c>
-      <c r="E44" t="s">
-        <v>37</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="G44" t="s">
-        <v>210</v>
-      </c>
-      <c r="M44" t="s">
-        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2272,47 +2312,49 @@
     <hyperlink ref="F11" r:id="rId13" xr:uid="{B82A3773-D31F-F745-8074-32333A4B6B5B}"/>
     <hyperlink ref="F12" r:id="rId14" xr:uid="{A07079BA-841D-FA42-873B-CC4775C0DCCC}"/>
     <hyperlink ref="E12" r:id="rId15" xr:uid="{BB3BABA2-AB59-C146-8AA3-33F0878C5102}"/>
-    <hyperlink ref="F15" r:id="rId16" xr:uid="{D019B855-B1D6-2040-9C70-A9DF1B7EA60F}"/>
-    <hyperlink ref="F16" r:id="rId17" xr:uid="{5CE2EE0D-7D5E-1048-A313-89538886CEF7}"/>
-    <hyperlink ref="F17" r:id="rId18" xr:uid="{56E9B766-594F-5948-9DF9-DCF2AD4E258D}"/>
-    <hyperlink ref="F18" r:id="rId19" xr:uid="{D321576E-4421-7C4F-9BC4-73015539CA4F}"/>
-    <hyperlink ref="E18" r:id="rId20" xr:uid="{7D281585-D3FA-5D47-AAD1-A60A5E792107}"/>
+    <hyperlink ref="F16" r:id="rId16" xr:uid="{D019B855-B1D6-2040-9C70-A9DF1B7EA60F}"/>
+    <hyperlink ref="F17" r:id="rId17" xr:uid="{5CE2EE0D-7D5E-1048-A313-89538886CEF7}"/>
+    <hyperlink ref="F18" r:id="rId18" xr:uid="{56E9B766-594F-5948-9DF9-DCF2AD4E258D}"/>
+    <hyperlink ref="F19" r:id="rId19" xr:uid="{D321576E-4421-7C4F-9BC4-73015539CA4F}"/>
+    <hyperlink ref="E19" r:id="rId20" xr:uid="{7D281585-D3FA-5D47-AAD1-A60A5E792107}"/>
     <hyperlink ref="E11" r:id="rId21" xr:uid="{C28378FE-16D5-CC4F-A7E3-71B6EC6253BF}"/>
-    <hyperlink ref="F19" r:id="rId22" xr:uid="{F34655E0-CD65-7A48-A686-9AAAAC4CEC48}"/>
-    <hyperlink ref="E20" r:id="rId23" xr:uid="{D8DBB0AD-F4FD-C343-9F24-39A7C0799653}"/>
-    <hyperlink ref="F21" r:id="rId24" xr:uid="{B10CE94D-5D47-9A4A-9332-9BE0837FEEDA}"/>
-    <hyperlink ref="F22" r:id="rId25" xr:uid="{610BC13E-92B8-504F-8A04-45B94B47CBF8}"/>
-    <hyperlink ref="E22" r:id="rId26" xr:uid="{4DE52B95-CE92-A745-B0BE-5B0A3679987E}"/>
-    <hyperlink ref="F23" r:id="rId27" xr:uid="{DF69D150-9965-104A-940F-471F1698665A}"/>
-    <hyperlink ref="F24" r:id="rId28" xr:uid="{D68304F9-6014-5D4C-8C51-2E6C594D3D4F}"/>
-    <hyperlink ref="F25" r:id="rId29" xr:uid="{A306D946-4621-434C-B4B4-EFC16BC8EFEB}"/>
-    <hyperlink ref="F26" r:id="rId30" xr:uid="{0A03C30E-833D-7B4A-B4E8-A0A603B4E141}"/>
-    <hyperlink ref="E26" r:id="rId31" xr:uid="{403F8941-ACA9-C94D-887C-E96D25747699}"/>
-    <hyperlink ref="F27" r:id="rId32" xr:uid="{512DF8DB-1848-7542-B778-6CDF38B3CA39}"/>
-    <hyperlink ref="E27" r:id="rId33" xr:uid="{8CAC1531-3736-F54A-BB96-58284FA3351B}"/>
-    <hyperlink ref="F28" r:id="rId34" xr:uid="{203A9358-D9CC-504F-9A1F-0F77D6A9546F}"/>
-    <hyperlink ref="F29" r:id="rId35" xr:uid="{99132808-6AC8-E442-9687-A11076E8FD47}"/>
-    <hyperlink ref="F30" r:id="rId36" xr:uid="{5671814E-4F6E-0342-AF28-02C384D5A6A4}"/>
-    <hyperlink ref="E30" r:id="rId37" xr:uid="{8964F743-296A-E349-AC76-4700BE7DCD51}"/>
-    <hyperlink ref="F31" r:id="rId38" xr:uid="{34FC6762-1B66-154B-8BB2-170D16F15629}"/>
-    <hyperlink ref="F32" r:id="rId39" xr:uid="{4EF2A7CB-6F4B-1443-93E1-B910D931DF14}"/>
-    <hyperlink ref="E32" r:id="rId40" xr:uid="{CD76C448-530E-3949-9D1B-ECBC6359302A}"/>
-    <hyperlink ref="F33" r:id="rId41" xr:uid="{5107AB5D-D49C-294A-AE13-A983380414A1}"/>
-    <hyperlink ref="E33" r:id="rId42" xr:uid="{424FD234-186B-4149-9599-5D04B3EAFD3C}"/>
-    <hyperlink ref="F34" r:id="rId43" xr:uid="{B6B2149E-5C67-C84A-BEEE-20481FF74448}"/>
-    <hyperlink ref="F36" r:id="rId44" xr:uid="{D132CCF7-CBF0-D946-B351-D3E77AD98205}"/>
-    <hyperlink ref="F35" r:id="rId45" xr:uid="{512770AB-A121-E94A-865A-9CE0E628EAF2}"/>
-    <hyperlink ref="F37" r:id="rId46" xr:uid="{5518BF54-1F92-5843-9EE5-5D8CFFBC3ED5}"/>
-    <hyperlink ref="F38" r:id="rId47" xr:uid="{7AE70F4A-F116-B840-8066-71BAC59FE161}"/>
-    <hyperlink ref="F39" r:id="rId48" xr:uid="{E35A1D4F-538C-EE4C-A048-59EA601B2A28}"/>
-    <hyperlink ref="F40" r:id="rId49" xr:uid="{AD67E94E-1D52-2044-AA01-D2B537426536}"/>
-    <hyperlink ref="F41" r:id="rId50" xr:uid="{0FFAFFC7-083F-9F4B-BDF9-0F734D9574DC}"/>
-    <hyperlink ref="F42" r:id="rId51" xr:uid="{42692C24-9D16-C84B-964F-74628EC3559A}"/>
-    <hyperlink ref="F43" r:id="rId52" xr:uid="{42147E18-CDF6-5D4C-9C2F-7FA6D2B033BB}"/>
-    <hyperlink ref="F44" r:id="rId53" xr:uid="{69726CBA-70F2-E847-A83E-2E8D5E2E6C14}"/>
+    <hyperlink ref="F20" r:id="rId22" xr:uid="{F34655E0-CD65-7A48-A686-9AAAAC4CEC48}"/>
+    <hyperlink ref="E21" r:id="rId23" xr:uid="{D8DBB0AD-F4FD-C343-9F24-39A7C0799653}"/>
+    <hyperlink ref="F22" r:id="rId24" xr:uid="{B10CE94D-5D47-9A4A-9332-9BE0837FEEDA}"/>
+    <hyperlink ref="F23" r:id="rId25" xr:uid="{610BC13E-92B8-504F-8A04-45B94B47CBF8}"/>
+    <hyperlink ref="E23" r:id="rId26" xr:uid="{4DE52B95-CE92-A745-B0BE-5B0A3679987E}"/>
+    <hyperlink ref="F24" r:id="rId27" xr:uid="{DF69D150-9965-104A-940F-471F1698665A}"/>
+    <hyperlink ref="F25" r:id="rId28" xr:uid="{D68304F9-6014-5D4C-8C51-2E6C594D3D4F}"/>
+    <hyperlink ref="F26" r:id="rId29" xr:uid="{A306D946-4621-434C-B4B4-EFC16BC8EFEB}"/>
+    <hyperlink ref="F27" r:id="rId30" xr:uid="{0A03C30E-833D-7B4A-B4E8-A0A603B4E141}"/>
+    <hyperlink ref="E27" r:id="rId31" xr:uid="{403F8941-ACA9-C94D-887C-E96D25747699}"/>
+    <hyperlink ref="F28" r:id="rId32" xr:uid="{512DF8DB-1848-7542-B778-6CDF38B3CA39}"/>
+    <hyperlink ref="E28" r:id="rId33" xr:uid="{8CAC1531-3736-F54A-BB96-58284FA3351B}"/>
+    <hyperlink ref="F29" r:id="rId34" xr:uid="{203A9358-D9CC-504F-9A1F-0F77D6A9546F}"/>
+    <hyperlink ref="F30" r:id="rId35" xr:uid="{99132808-6AC8-E442-9687-A11076E8FD47}"/>
+    <hyperlink ref="F31" r:id="rId36" xr:uid="{5671814E-4F6E-0342-AF28-02C384D5A6A4}"/>
+    <hyperlink ref="E31" r:id="rId37" xr:uid="{8964F743-296A-E349-AC76-4700BE7DCD51}"/>
+    <hyperlink ref="F32" r:id="rId38" xr:uid="{34FC6762-1B66-154B-8BB2-170D16F15629}"/>
+    <hyperlink ref="F33" r:id="rId39" xr:uid="{4EF2A7CB-6F4B-1443-93E1-B910D931DF14}"/>
+    <hyperlink ref="E33" r:id="rId40" xr:uid="{CD76C448-530E-3949-9D1B-ECBC6359302A}"/>
+    <hyperlink ref="F34" r:id="rId41" xr:uid="{5107AB5D-D49C-294A-AE13-A983380414A1}"/>
+    <hyperlink ref="E34" r:id="rId42" xr:uid="{424FD234-186B-4149-9599-5D04B3EAFD3C}"/>
+    <hyperlink ref="F35" r:id="rId43" xr:uid="{B6B2149E-5C67-C84A-BEEE-20481FF74448}"/>
+    <hyperlink ref="F37" r:id="rId44" xr:uid="{D132CCF7-CBF0-D946-B351-D3E77AD98205}"/>
+    <hyperlink ref="F36" r:id="rId45" xr:uid="{512770AB-A121-E94A-865A-9CE0E628EAF2}"/>
+    <hyperlink ref="F38" r:id="rId46" xr:uid="{5518BF54-1F92-5843-9EE5-5D8CFFBC3ED5}"/>
+    <hyperlink ref="F39" r:id="rId47" xr:uid="{7AE70F4A-F116-B840-8066-71BAC59FE161}"/>
+    <hyperlink ref="F40" r:id="rId48" xr:uid="{E35A1D4F-538C-EE4C-A048-59EA601B2A28}"/>
+    <hyperlink ref="F41" r:id="rId49" xr:uid="{AD67E94E-1D52-2044-AA01-D2B537426536}"/>
+    <hyperlink ref="F42" r:id="rId50" xr:uid="{0FFAFFC7-083F-9F4B-BDF9-0F734D9574DC}"/>
+    <hyperlink ref="F43" r:id="rId51" xr:uid="{42692C24-9D16-C84B-964F-74628EC3559A}"/>
+    <hyperlink ref="F44" r:id="rId52" xr:uid="{42147E18-CDF6-5D4C-9C2F-7FA6D2B033BB}"/>
+    <hyperlink ref="F45" r:id="rId53" xr:uid="{69726CBA-70F2-E847-A83E-2E8D5E2E6C14}"/>
     <hyperlink ref="F13" r:id="rId54" xr:uid="{7448DAB6-7FFF-FF4F-8C76-987F18113B3B}"/>
     <hyperlink ref="F14" r:id="rId55" xr:uid="{7476ACCC-D963-4141-916F-84E6366DB338}"/>
     <hyperlink ref="E14" r:id="rId56" xr:uid="{78D50B19-5159-284F-B66D-DB467686A7D8}"/>
+    <hyperlink ref="F15" r:id="rId57" xr:uid="{387E7003-A1B4-CF46-9BD3-CB3474E4E668}"/>
+    <hyperlink ref="E15" r:id="rId58" xr:uid="{794AA027-79EC-964A-A5D1-BA2E907B7327}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>